<commit_message>
memoria: auto-refresh resumo + dashboard (18:15 task)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/memoria/memoria-resumo.xlsx
+++ b/memoria/memoria-resumo.xlsx
@@ -3808,10 +3808,10 @@
         <v>1120</v>
       </c>
       <c r="I7" t="n">
-        <v>865.73</v>
+        <v>861</v>
       </c>
       <c r="J7" t="n">
-        <v>163.77</v>
+        <v>163.61</v>
       </c>
     </row>
     <row r="8">
@@ -3842,10 +3842,10 @@
         <v>728</v>
       </c>
       <c r="I8" t="n">
-        <v>1466000</v>
+        <v>1418000</v>
       </c>
       <c r="J8" t="n">
-        <v>580750.16</v>
+        <v>574122.8</v>
       </c>
     </row>
     <row r="9">
@@ -3876,7 +3876,7 @@
         <v>5969</v>
       </c>
       <c r="I9" t="n">
-        <v>235000</v>
+        <v>231500</v>
       </c>
       <c r="J9" t="n">
         <v>75198.12</v>
@@ -3910,10 +3910,10 @@
         <v>540</v>
       </c>
       <c r="I10" t="n">
-        <v>47730</v>
+        <v>48010</v>
       </c>
       <c r="J10" t="n">
-        <v>13503.49</v>
+        <v>13532.64</v>
       </c>
     </row>
     <row r="11">
@@ -3944,10 +3944,10 @@
         <v>145</v>
       </c>
       <c r="I11" t="n">
-        <v>1215.98</v>
+        <v>1237.92</v>
       </c>
       <c r="J11" t="n">
-        <v>237.45</v>
+        <v>237.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>